<commit_message>
fix(privacy): redact public exports and restrict Netlify output
- export_bookings_excel.py redacts customer phone numbers by default (booked
  slots show only the 'محجوز' marker); --no-redact is opt-in for private runs.
  The already-committed public workbook was redacted in place (4 phone cells
  removed; 0 phone-shaped values remain). Owner history-purge steps documented
  in docs/OWNER_PII_CLEANUP.md (not run automatically).
- netlify.toml + scripts/build-netlify.mjs publish only the app files
  (index.html/404.html/icon.svg/.nojekyll) so Netlify can no longer serve
  exports/, database/, docs/, tests/, scripts/ or the Supabase functions.
  GitHub Pages is unaffected.
- tests unzip the produced workbook (no PII patterns) and inspect the Netlify
  publish dir (no exports/private files).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vA9n14SRKu5UrMT2X1E9z
</commit_message>
<xml_diff>
--- a/exports/bookings-2026.xlsx
+++ b/exports/bookings-2026.xlsx
@@ -9221,7 +9221,7 @@
       </c>
       <c r="N260" s="20" t="inlineStr">
         <is>
-          <t>0503666853</t>
+          <t>محجوز</t>
         </is>
       </c>
       <c r="O260" s="21" t="n">
@@ -9306,7 +9306,7 @@
       </c>
       <c r="H263" s="51" t="inlineStr">
         <is>
-          <t>‪+966549031970‬</t>
+          <t>محجوز</t>
         </is>
       </c>
       <c r="I263" s="51" t="n">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="E264" s="52" t="inlineStr">
         <is>
-          <t>‪+966 55 969 6330‬</t>
+          <t>محجوز</t>
         </is>
       </c>
       <c r="F264" s="53" t="n">
@@ -10166,7 +10166,7 @@
       </c>
       <c r="H291" s="51" t="inlineStr">
         <is>
-          <t>+966 54 556 9050</t>
+          <t>محجوز</t>
         </is>
       </c>
       <c r="I291" s="51" t="n">

</xml_diff>